<commit_message>
Test Mr. Advocate's second review: section subjects confirmed; Act-specific plain-language phrases added to N2; one leading case (Satish Chander Ahuja) is not in the index
Of his 82 phrases the intended Act fires on 11/27, 22/31, 16/24 under N2 with no cross-Act firing; used questions unchanged. Graded boost not adopted.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01YEUNXbYb9LDbJLc2ziqL3n
</commit_message>
<xml_diff>
--- a/review_data/ruler/inputs/2026-10-12_trigger_workbook_with_spec_v2.xlsx
+++ b/review_data/ruler/inputs/2026-10-12_trigger_workbook_with_spec_v2.xlsx
@@ -1635,7 +1635,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C20"/>
+  <dimension ref="A1:C21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="44" customWidth="1" style="44" min="1" max="1"/>
@@ -1901,7 +1901,7 @@
       </c>
       <c r="C17" s="65" t="inlineStr">
         <is>
-          <t>59 question cases (N1 and N2 each), 26 passage cases, 2 label tests: all pass after fixing two patterns and correcting three of my own wrong expectations. Not a lawyer's test.</t>
+          <t>70 question cases (N1 and N2 each), 26 passage cases, 2 label tests: all pass after fixing patterns and correcting three of my own wrong expectations. Not a lawyer's test.</t>
         </is>
       </c>
     </row>
@@ -1942,11 +1942,28 @@
     <row r="20">
       <c r="A20" s="65" t="inlineStr">
         <is>
+          <t>Mr. Advocate's second review (section-by-section triggers for PWDVA, NDPS, UAPA), 2026-10-12</t>
+        </is>
+      </c>
+      <c r="B20" s="65" t="inlineStr">
+        <is>
+          <t>Confirms the section subjects for these 3 Acts; supplies 82 plain-language phrases and 9 leading cases</t>
+        </is>
+      </c>
+      <c r="C20" s="65" t="inlineStr">
+        <is>
+          <t>Plain-language tier (N2) extended with the Act-specific phrases only: evict/throw out with in-laws or husband, matrimonial home with a right/stay word, abusive husband or partner, emotional abuse with a family word, breach of a protection order; drugs near police/found/bag/caught/search words (with medical/forensic exclusions); 'banned our organisation', separatist with arrest/support words. Not added: phrases with no Act cue (e.g. 'Can I get another place to live?', 'Police searched my body'), which are exactly the look-alike ambiguity the test is about. Of his 82 phrases the intended Act now fires on 11 of 27 (PWDVA), 22 of 31 (NDPS), 16 of 24 (UAPA) under N2 (4, 3, 4 under N1); no phrase fires a different Act; the 30 used questions are unchanged (N1 7, N2 11). The recall figures are optimistic because the additions were written from the same phrases.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="65" t="inlineStr">
+        <is>
           <t>Open for Mr. Advocate</t>
         </is>
       </c>
-      <c r="B20" s="65" t="inlineStr"/>
-      <c r="C20" s="65" t="inlineStr">
+      <c r="B21" s="65" t="inlineStr"/>
+      <c r="C21" s="65" t="inlineStr">
         <is>
           <t>(1) Are the section lists right (e.g. PWDVA 12,17-23,31; NDPS 20-22,27A,29,37,42,43,50,52A,57,67; UAPA 10,13,15-18,20,38-40,43D,43E)? (2) Any exclusion or anchor that would misfire in a real client's words? (3) Is a bare 'Domestic Violence Act' and 'Juvenile Justice Act' (including the 1986 and 2000 Acts) acceptable as markers?</t>
         </is>
@@ -5482,7 +5499,7 @@
     <row r="1">
       <c r="A1" s="83" t="inlineStr">
         <is>
-          <t>MACHINE SPEC v2 (DRAFT 2026-10-12; not frozen). Source of truth: review_tools/machine_spec_v2.py; JSON export review_data/ruler/machine_spec_v2.json, sha256 634547e68c200257... Flags: case-insensitive, DOTALL; acronyms case-sensitive via (?-i:...); near(a,b,n) = a within n characters of b in either order (written out in full below). N1 = precise question anchors (Mr. Advocate's, repaired). N2 = N1 or the plain-language anchors, unless the Act's exclusion pattern matches the question. Passage markers are shared by N1 and N2.</t>
+          <t>MACHINE SPEC v2 (DRAFT 2026-10-12; not frozen). Source of truth: review_tools/machine_spec_v2.py; JSON export review_data/ruler/machine_spec_v2.json, sha256 ca9afa8c3c42c926... Flags: case-insensitive, DOTALL; acronyms case-sensitive via (?-i:...); near(a,b,n) = a within n characters of b in either order (written out in full below). N1 = precise question anchors (Mr. Advocate's, repaired). N2 = N1 or the plain-language anchors, unless the Act's exclusion pattern matches the question. Passage markers are shared by N1 and N2.</t>
         </is>
       </c>
     </row>
@@ -5539,7 +5556,12 @@
 2. \bfamily violence\b
 3. \b(?:threw|thrown|throw|throws|throwing|kicked|drove|driven)\s+(?:me|her|us|my wife|his wife)\s+out of\s+(?:the |my |our |his )?(?:marital |matrimonial |shared )?(?:house|home)\b
 4. \b(?:husband|in-?laws?|mother-in-law|partner|boyfriend)\b.{0,30}\b(?:hits?|beats?|beat|beating|abus\w+|tortur\w+|harass\w+|threaten\w*)\s+(?:me|her)\b
-5. \bright to (?:stay|live|reside) in (?:the|my|our) (?:house|home)\b</t>
+5. \bright to (?:stay|live|reside) in (?:the|my|our) (?:house|home)\b
+6. (?:(?:\b(?:evict\w*|throw\w*\s+(?:me\s+)?out|kick\w*\s+(?:me\s+)?out)\b).{0,60}(?:\b(?:in-?laws?|husband|matrimonial|marital|mother-in-law)\b)|(?:\b(?:in-?laws?|husband|matrimonial|marital|mother-in-law)\b).{0,60}(?:\b(?:evict\w*|throw\w*\s+(?:me\s+)?out|kick\w*\s+(?:me\s+)?out)\b))
+7. (?:(?:\b(?:matrimonial|marital) home\b).{0,60}(?:\b(?:right|stay|live|reside|evict\w*|throw\w*|name)\b)|(?:\b(?:right|stay|live|reside|evict\w*|throw\w*|name)\b).{0,60}(?:\b(?:matrimonial|marital) home\b))
+8. \b(?:abusive|violent)\s+(?:husband|partner|boyfriend|spouse)\b
+9. (?:(?:\b(?:emotional|mental|physical|verbal)\s+(?:abuse|torture)\b).{0,80}(?:\b(?:husband|wife|partner|in-?laws?|home|house)\b)|(?:\b(?:husband|wife|partner|in-?laws?|home|house)\b).{0,80}(?:\b(?:emotional|mental|physical|verbal)\s+(?:abuse|torture)\b))
+10. (?:(?:\bprotection order\b).{0,40}(?:\b(?:broke|broken|breach\w*|violat\w*)\b)|(?:\b(?:broke|broken|breach\w*|violat\w*)\b).{0,40}(?:\bprotection order\b))</t>
         </is>
       </c>
       <c r="D4" s="65" t="inlineStr">
@@ -5582,12 +5604,13 @@
           <t>1. (?:(?:\b(?:ganja|charas|hashish|heroin|cocaine|MDMA|methamphetamine|opium|poppy husk|poppy straw|smack|brown sugar|marijuana|cannabis|ecstasy|LSD|tramadol|codeine)\b).{0,80}(?:\b(?:found|caught|arrest\w*|police|NCB|bag|car|room|carry\w*|sell\w*|sold|peddl\w+|smuggl\w+|bail|statement)\b)|(?:\b(?:found|caught|arrest\w*|police|NCB|bag|car|room|carry\w*|sell\w*|sold|peddl\w+|smuggl\w+|bail|statement)\b).{0,80}(?:\b(?:ganja|charas|hashish|heroin|cocaine|MDMA|methamphetamine|opium|poppy husk|poppy straw|smack|brown sugar|marijuana|cannabis|ecstasy|LSD|tramadol|codeine)\b))
 2. (?-i:\bNCB\b)
 3. \bnarcotics?\b
-4. (?:(?:\b(?:drug|drugs)\b).{0,40}(?:\b(?:case|peddling|trafficking|dealer|smuggling|bail|seized|caught)\b)|(?:\b(?:case|peddling|trafficking|dealer|smuggling|bail|seized|caught)\b).{0,40}(?:\b(?:drug|drugs)\b))</t>
+4. (?:(?:\b(?:drug|drugs)\b).{0,40}(?:\b(?:case|peddling|trafficking|dealer|smuggling|bail|seized|caught)\b)|(?:\b(?:case|peddling|trafficking|dealer|smuggling|bail|seized|caught)\b).{0,40}(?:\b(?:drug|drugs)\b))
+5. (?:(?:\b(?:drug|drugs|narcotic\w*|contraband|illegal tablets?|illegal pills?)\b).{0,80}(?:\b(?:police|find|found|bag|arrested|caught|seized|carrying|search\w*|funded|delivery|gang|tip|confess\w*|admit\w*|samples?|seizure|magistrate|gazetted)\b)|(?:\b(?:police|find|found|bag|arrested|caught|seized|carrying|search\w*|funded|delivery|gang|tip|confess\w*|admit\w*|samples?|seizure|magistrate|gazetted)\b).{0,80}(?:\b(?:drug|drugs|narcotic\w*|contraband|illegal tablets?|illegal pills?)\b))</t>
         </is>
       </c>
       <c r="D5" s="65" t="inlineStr">
         <is>
-          <t>\b(?:forensic|toxicolog\w*|post-?mortem|autopsy|traces? of|prescri\w+|pharmacy|medicine)\b</t>
+          <t>\b(?:forensic|toxicolog\w*|post-?mortem|autopsy|traces? of|prescri\w+|pharmacy|medicine|doctor|hospital|patient|treatment|illness|fever)\b</t>
         </is>
       </c>
       <c r="E5" s="65" t="inlineStr">
@@ -5773,8 +5796,9 @@
         <is>
           <t>1. \banti[- ]terror (?:law|act)\b
 2. (?:(?:\bterror\w*).{0,60}(?:\b(?:booked|arrested|accused|charged|FIR|bail|case)\b)|(?:\b(?:booked|arrested|accused|charged|FIR|bail|case)\b).{0,60}(?:\bterror\w*))
-3. \bbanned (?:organi[sz]ation|group)\b
-4. \bterror funding\b</t>
+3. \bbanned\s+(?:our\s+|the\s+|an?\s+)?(?:organi[sz]ation|group|association)\b
+4. \bterror funding\b
+5. (?:(?:\b(?:separatist|unlawful association)\b).{0,60}(?:\b(?:arrest\w*|accused|booked|supporting|member\w*|belong\w*|links?)\b)|(?:\b(?:arrest\w*|accused|booked|supporting|member\w*|belong\w*|links?)\b).{0,60}(?:\b(?:separatist|unlawful association)\b))</t>
         </is>
       </c>
       <c r="D10" s="65" t="inlineStr">

</xml_diff>